<commit_message>
feat(buqi): unify demo text in Chinese
</commit_message>
<xml_diff>
--- a/Design/Excel/GameHot/Datas/Buqi/BuqiEvent.xlsx
+++ b/Design/Excel/GameHot/Datas/Buqi/BuqiEvent.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BuqiEvent" sheetId="1" r:id="R03d950f866484ab4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BuqiEvent" sheetId="1" r:id="R7659e0470bd94eec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -390,7 +390,7 @@
         <x:v>event-trial-stele</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>试锋碑</x:v>
+        <x:v>攻击测试碑 · 试锋</x:v>
       </x:c>
       <x:c r="D4" t="str">
         <x:v>Buqi.Content.Event.event_trial_stele.Name</x:v>
@@ -404,9 +404,9 @@
       <x:c r="G4" t="n">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="H4" t="str"/>
-      <x:c r="I4" t="str"/>
-      <x:c r="J4" t="str"/>
+      <x:c r="H4"/>
+      <x:c r="I4"/>
+      <x:c r="J4"/>
       <x:c r="K4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -423,7 +423,7 @@
         <x:v>event-herb-stall</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>旧城药摊</x:v>
+        <x:v>恢复药摊 · 旧城</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Buqi.Content.Event.event_herb_stall.Name</x:v>
@@ -437,9 +437,9 @@
       <x:c r="G5" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="H5" t="str"/>
-      <x:c r="I5" t="str"/>
-      <x:c r="J5" t="str"/>
+      <x:c r="H5"/>
+      <x:c r="I5"/>
+      <x:c r="J5"/>
       <x:c r="K5" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -456,7 +456,7 @@
         <x:v>event-broken-armor</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>山门残甲</x:v>
+        <x:v>护盾装备 · 山门残甲</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Buqi.Content.Event.event_broken_armor.Name</x:v>
@@ -470,9 +470,9 @@
       <x:c r="G6" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="H6" t="str"/>
-      <x:c r="I6" t="str"/>
-      <x:c r="J6" t="str"/>
+      <x:c r="H6"/>
+      <x:c r="I6"/>
+      <x:c r="J6"/>
       <x:c r="K6" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -489,7 +489,7 @@
         <x:v>event-cloud-peddler</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>云脚行商</x:v>
+        <x:v>旅行商人 · 云脚</x:v>
       </x:c>
       <x:c r="D7" t="str">
         <x:v>Buqi.Content.Event.event_cloud_peddler.Name</x:v>
@@ -503,9 +503,9 @@
       <x:c r="G7" t="n">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="H7" t="str"/>
-      <x:c r="I7" t="str"/>
-      <x:c r="J7" t="str"/>
+      <x:c r="H7"/>
+      <x:c r="I7"/>
+      <x:c r="J7"/>
       <x:c r="K7" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -522,7 +522,7 @@
         <x:v>event-borrowed-flame</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>借火炼器</x:v>
+        <x:v>强化炉 · 借火</x:v>
       </x:c>
       <x:c r="D8" t="str">
         <x:v>Buqi.Content.Event.event_borrowed_flame.Name</x:v>
@@ -536,7 +536,7 @@
       <x:c r="G8" t="n">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="H8" t="str"/>
+      <x:c r="H8"/>
       <x:c r="I8" t="str">
         <x:v>borrowed_flame</x:v>
       </x:c>
@@ -559,7 +559,7 @@
         <x:v>event-broken-mechanism</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>断弦机括</x:v>
+        <x:v>损坏机关 · 断弦</x:v>
       </x:c>
       <x:c r="D9" t="str">
         <x:v>Buqi.Content.Event.event_broken_mechanism.Name</x:v>
@@ -573,9 +573,9 @@
       <x:c r="G9" t="n">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="H9" t="str"/>
-      <x:c r="I9" t="str"/>
-      <x:c r="J9" t="str"/>
+      <x:c r="H9"/>
+      <x:c r="I9"/>
+      <x:c r="J9"/>
       <x:c r="K9" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -592,7 +592,7 @@
         <x:v>event-nameless-ledger</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>无名账册</x:v>
+        <x:v>金币账册 · 无名</x:v>
       </x:c>
       <x:c r="D10" t="str">
         <x:v>Buqi.Content.Event.event_nameless_ledger.Name</x:v>
@@ -606,7 +606,7 @@
       <x:c r="G10" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="H10" t="str"/>
+      <x:c r="H10"/>
       <x:c r="I10" t="str">
         <x:v>ledger_owed|ledger_closed</x:v>
       </x:c>
@@ -629,7 +629,7 @@
         <x:v>event-rain-umbrella</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>雨夜借伞</x:v>
+        <x:v>护盾雨伞 · 雨夜</x:v>
       </x:c>
       <x:c r="D11" t="str">
         <x:v>Buqi.Content.Event.event_rain_umbrella.Name</x:v>
@@ -643,7 +643,7 @@
       <x:c r="G11" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="H11" t="str"/>
+      <x:c r="H11"/>
       <x:c r="I11" t="str">
         <x:v>umbrella_borrowed|umbrella_returned</x:v>
       </x:c>
@@ -666,7 +666,7 @@
         <x:v>event-sword-echo</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>剑痕回声</x:v>
+        <x:v>攻击记录 · 剑痕</x:v>
       </x:c>
       <x:c r="D12" t="str">
         <x:v>Buqi.Content.Event.event_sword_echo.Name</x:v>
@@ -680,9 +680,9 @@
       <x:c r="G12" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="H12" t="str"/>
-      <x:c r="I12" t="str"/>
-      <x:c r="J12" t="str"/>
+      <x:c r="H12"/>
+      <x:c r="I12"/>
+      <x:c r="J12"/>
       <x:c r="K12" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -699,7 +699,7 @@
         <x:v>event-wall-fissure</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>城墙裂隙</x:v>
+        <x:v>护盾挑战 · 城墙裂隙</x:v>
       </x:c>
       <x:c r="D13" t="str">
         <x:v>Buqi.Content.Event.event_wall_fissure.Name</x:v>
@@ -713,9 +713,9 @@
       <x:c r="G13" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="H13" t="str"/>
-      <x:c r="I13" t="str"/>
-      <x:c r="J13" t="str"/>
+      <x:c r="H13"/>
+      <x:c r="I13"/>
+      <x:c r="J13"/>
       <x:c r="K13" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -732,7 +732,7 @@
         <x:v>event-herb-water</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>药田争水</x:v>
+        <x:v>恢复训练 · 药田争水</x:v>
       </x:c>
       <x:c r="D14" t="str">
         <x:v>Buqi.Content.Event.event_herb_water.Name</x:v>
@@ -746,9 +746,9 @@
       <x:c r="G14" t="n">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="H14" t="str"/>
-      <x:c r="I14" t="str"/>
-      <x:c r="J14" t="str"/>
+      <x:c r="H14"/>
+      <x:c r="I14"/>
+      <x:c r="J14"/>
       <x:c r="K14" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -765,7 +765,7 @@
         <x:v>event-roving-furnace</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>游炉换火</x:v>
+        <x:v>强化炉 · 换火</x:v>
       </x:c>
       <x:c r="D15" t="str">
         <x:v>Buqi.Content.Event.event_roving_furnace.Name</x:v>
@@ -782,8 +782,8 @@
       <x:c r="H15" t="str">
         <x:v>borrowed_flame</x:v>
       </x:c>
-      <x:c r="I15" t="str"/>
-      <x:c r="J15" t="str"/>
+      <x:c r="I15"/>
+      <x:c r="J15"/>
       <x:c r="K15" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -800,7 +800,7 @@
         <x:v>event-ledger-collector</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>欠账来客</x:v>
+        <x:v>欠款结算 · 来客</x:v>
       </x:c>
       <x:c r="D16" t="str">
         <x:v>Buqi.Content.Event.event_ledger_collector.Name</x:v>
@@ -817,8 +817,8 @@
       <x:c r="H16" t="str">
         <x:v>ledger_owed</x:v>
       </x:c>
-      <x:c r="I16" t="str"/>
-      <x:c r="J16" t="str"/>
+      <x:c r="I16"/>
+      <x:c r="J16"/>
       <x:c r="K16" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -835,7 +835,7 @@
         <x:v>event-umbrella-return</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>归伞人</x:v>
+        <x:v>护盾雨伞 · 归还</x:v>
       </x:c>
       <x:c r="D17" t="str">
         <x:v>Buqi.Content.Event.event_umbrella_return.Name</x:v>
@@ -852,8 +852,8 @@
       <x:c r="H17" t="str">
         <x:v>umbrella_borrowed</x:v>
       </x:c>
-      <x:c r="I17" t="str"/>
-      <x:c r="J17" t="str"/>
+      <x:c r="I17"/>
+      <x:c r="J17"/>
       <x:c r="K17" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -870,7 +870,7 @@
         <x:v>event-headwind-array</x:v>
       </x:c>
       <x:c r="C18" t="str">
-        <x:v>逆风试阵</x:v>
+        <x:v>加速挑战 · 逆风</x:v>
       </x:c>
       <x:c r="D18" t="str">
         <x:v>Buqi.Content.Event.event_headwind_array.Name</x:v>
@@ -884,9 +884,9 @@
       <x:c r="G18" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="H18" t="str"/>
-      <x:c r="I18" t="str"/>
-      <x:c r="J18" t="str"/>
+      <x:c r="H18"/>
+      <x:c r="I18"/>
+      <x:c r="J18"/>
       <x:c r="K18" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -903,7 +903,7 @@
         <x:v>event-three-bidders</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>三家竞价</x:v>
+        <x:v>装备竞价 · 三家</x:v>
       </x:c>
       <x:c r="D19" t="str">
         <x:v>Buqi.Content.Event.event_three_bidders.Name</x:v>
@@ -917,7 +917,7 @@
       <x:c r="G19" t="n">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="H19" t="str"/>
+      <x:c r="H19"/>
       <x:c r="I19" t="str">
         <x:v>auction_claim</x:v>
       </x:c>
@@ -940,7 +940,7 @@
         <x:v>event-heaven-gate</x:v>
       </x:c>
       <x:c r="C20" t="str">
-        <x:v>天门校器</x:v>
+        <x:v>攻击校准 · 天门</x:v>
       </x:c>
       <x:c r="D20" t="str">
         <x:v>Buqi.Content.Event.event_heaven_gate.Name</x:v>
@@ -954,9 +954,9 @@
       <x:c r="G20" t="n">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="H20" t="str"/>
-      <x:c r="I20" t="str"/>
-      <x:c r="J20" t="str"/>
+      <x:c r="H20"/>
+      <x:c r="I20"/>
+      <x:c r="J20"/>
       <x:c r="K20" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -973,7 +973,7 @@
         <x:v>event-mountain-eye</x:v>
       </x:c>
       <x:c r="C21" t="str">
-        <x:v>护山阵眼</x:v>
+        <x:v>护盾核心 · 护山</x:v>
       </x:c>
       <x:c r="D21" t="str">
         <x:v>Buqi.Content.Event.event_mountain_eye.Name</x:v>
@@ -987,9 +987,9 @@
       <x:c r="G21" t="n">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="H21" t="str"/>
-      <x:c r="I21" t="str"/>
-      <x:c r="J21" t="str"/>
+      <x:c r="H21"/>
+      <x:c r="I21"/>
+      <x:c r="J21"/>
       <x:c r="K21" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1006,7 +1006,7 @@
         <x:v>event-herbs-return</x:v>
       </x:c>
       <x:c r="C22" t="str">
-        <x:v>百草归元</x:v>
+        <x:v>恢复强化 · 百草</x:v>
       </x:c>
       <x:c r="D22" t="str">
         <x:v>Buqi.Content.Event.event_herbs_return.Name</x:v>
@@ -1020,9 +1020,9 @@
       <x:c r="G22" t="n">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="H22" t="str"/>
-      <x:c r="I22" t="str"/>
-      <x:c r="J22" t="str"/>
+      <x:c r="H22"/>
+      <x:c r="I22"/>
+      <x:c r="J22"/>
       <x:c r="K22" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1039,7 +1039,7 @@
         <x:v>event-old-pacts</x:v>
       </x:c>
       <x:c r="C23" t="str">
-        <x:v>旧约清算</x:v>
+        <x:v>欠款清算 · 旧约</x:v>
       </x:c>
       <x:c r="D23" t="str">
         <x:v>Buqi.Content.Event.event_old_pacts.Name</x:v>
@@ -1053,9 +1053,9 @@
       <x:c r="G23" t="n">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="H23" t="str"/>
-      <x:c r="I23" t="str"/>
-      <x:c r="J23" t="str"/>
+      <x:c r="H23"/>
+      <x:c r="I23"/>
+      <x:c r="J23"/>
       <x:c r="K23" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1072,7 +1072,7 @@
         <x:v>event-scrap-recovery</x:v>
       </x:c>
       <x:c r="C24" t="str">
-        <x:v>回收残器</x:v>
+        <x:v>装备回收 · 残件</x:v>
       </x:c>
       <x:c r="D24" t="str">
         <x:v>Buqi.Content.Event.event_scrap_recovery.Name</x:v>
@@ -1086,9 +1086,9 @@
       <x:c r="G24" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="H24" t="str"/>
-      <x:c r="I24" t="str"/>
-      <x:c r="J24" t="str"/>
+      <x:c r="H24"/>
+      <x:c r="I24"/>
+      <x:c r="J24"/>
       <x:c r="K24" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1105,7 +1105,7 @@
         <x:v>event-calming-chime</x:v>
       </x:c>
       <x:c r="C25" t="str">
-        <x:v>镇心钟鸣</x:v>
+        <x:v>状态调整 · 钟鸣</x:v>
       </x:c>
       <x:c r="D25" t="str">
         <x:v>Buqi.Content.Event.event_calming_chime.Name</x:v>
@@ -1119,9 +1119,9 @@
       <x:c r="G25" t="n">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="H25" t="str"/>
-      <x:c r="I25" t="str"/>
-      <x:c r="J25" t="str"/>
+      <x:c r="H25"/>
+      <x:c r="I25"/>
+      <x:c r="J25"/>
       <x:c r="K25" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1138,7 +1138,7 @@
         <x:v>event-day-nine-ledger</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>九日归账</x:v>
+        <x:v>第九日结算 · 账单</x:v>
       </x:c>
       <x:c r="D26" t="str">
         <x:v>Buqi.Content.Event.event_day_nine_ledger.Name</x:v>
@@ -1155,8 +1155,8 @@
       <x:c r="H26" t="str">
         <x:v>auction_claim</x:v>
       </x:c>
-      <x:c r="I26" t="str"/>
-      <x:c r="J26" t="str"/>
+      <x:c r="I26"/>
+      <x:c r="J26"/>
       <x:c r="K26" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1173,7 +1173,7 @@
         <x:v>event-return-furnace</x:v>
       </x:c>
       <x:c r="C27" t="str">
-        <x:v>不器归炉</x:v>
+        <x:v>最终强化 · 不器归炉</x:v>
       </x:c>
       <x:c r="D27" t="str">
         <x:v>Buqi.Content.Event.event_return_furnace.Name</x:v>
@@ -1187,9 +1187,9 @@
       <x:c r="G27" t="n">
         <x:v>150</x:v>
       </x:c>
-      <x:c r="H27" t="str"/>
-      <x:c r="I27" t="str"/>
-      <x:c r="J27" t="str"/>
+      <x:c r="H27"/>
+      <x:c r="I27"/>
+      <x:c r="J27"/>
       <x:c r="K27" t="n">
         <x:v>0</x:v>
       </x:c>

</xml_diff>